<commit_message>
Update Meesho template version handling
</commit_message>
<xml_diff>
--- a/main/marketplaces/meesho/Sarees-10003-EXTERNAL-MeeshoTemplate2PricesGSTIN.xlsx
+++ b/main/marketplaces/meesho/Sarees-10003-EXTERNAL-MeeshoTemplate2PricesGSTIN.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10197" uniqueCount="4897">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10213" uniqueCount="4905">
   <si>
     <t>Return Reasons</t>
   </si>
@@ -5471,6 +5471,9 @@
     <t>Elbwear</t>
   </si>
   <si>
+    <t>Elegance fashion and style</t>
+  </si>
+  <si>
     <t>Ellestifab</t>
   </si>
   <si>
@@ -6656,6 +6659,9 @@
     <t>Hitesh Trendz</t>
   </si>
   <si>
+    <t>Hiyasilk</t>
+  </si>
+  <si>
     <t>Ho Bindaass</t>
   </si>
   <si>
@@ -7097,6 +7103,9 @@
     <t>JOMSO</t>
   </si>
   <si>
+    <t>JONEE SAREE</t>
+  </si>
+  <si>
     <t>JOVTY</t>
   </si>
   <si>
@@ -12095,6 +12104,12 @@
     <t>Shiv Fashion</t>
   </si>
   <si>
+    <t>Shiv Omm Collections</t>
+  </si>
+  <si>
+    <t>Shiv Textiles</t>
+  </si>
+  <si>
     <t>Shivam Creation</t>
   </si>
   <si>
@@ -14012,6 +14027,9 @@
     <t>Warthy Ent</t>
   </si>
   <si>
+    <t>Watch and Wear</t>
+  </si>
+  <si>
     <t>WavySnugsy</t>
   </si>
   <si>
@@ -14432,6 +14450,9 @@
     <t>aagza</t>
   </si>
   <si>
+    <t>abhi enterprise premium</t>
+  </si>
+  <si>
     <t>anbhiga</t>
   </si>
   <si>
@@ -14535,6 +14556,9 @@
   </si>
   <si>
     <t>inch pinch</t>
+  </si>
+  <si>
+    <t>iprise creation</t>
   </si>
   <si>
     <t>izkio</t>
@@ -18923,13 +18947,13 @@
         <v>10003.0</v>
       </c>
       <c r="C101" t="n" s="98">
-        <v>53.0</v>
+        <v>58.0</v>
       </c>
       <c r="D101" t="s" s="99">
-        <v>4896</v>
+        <v>4904</v>
       </c>
       <c r="E101" t="s" s="100">
-        <v>4896</v>
+        <v>4904</v>
       </c>
     </row>
     <row r="102" ht="15.75" customHeight="1"/>
@@ -21067,7 +21091,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:BA3963"/>
+  <dimension ref="A1:BA3971"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="2" max="2" width="23.4375" customWidth="true"/>
@@ -32282,22 +32306,22 @@
     </row>
     <row r="1642">
       <c r="AU1642" t="s" s="0">
-        <v>619</v>
+        <v>2512</v>
       </c>
     </row>
     <row r="1643">
       <c r="AU1643" t="s" s="0">
-        <v>2512</v>
+        <v>2513</v>
       </c>
     </row>
     <row r="1644">
       <c r="AU1644" t="s" s="0">
-        <v>2513</v>
+        <v>2514</v>
       </c>
     </row>
     <row r="1645">
       <c r="AU1645" t="s" s="0">
-        <v>2514</v>
+        <v>619</v>
       </c>
     </row>
     <row r="1646">
@@ -34097,22 +34121,22 @@
     </row>
     <row r="2005">
       <c r="AU2005" t="s" s="0">
-        <v>367</v>
+        <v>2874</v>
       </c>
     </row>
     <row r="2006">
       <c r="AU2006" t="s" s="0">
-        <v>2874</v>
+        <v>2875</v>
       </c>
     </row>
     <row r="2007">
       <c r="AU2007" t="s" s="0">
-        <v>2875</v>
+        <v>2876</v>
       </c>
     </row>
     <row r="2008">
       <c r="AU2008" t="s" s="0">
-        <v>2876</v>
+        <v>367</v>
       </c>
     </row>
     <row r="2009">
@@ -39352,22 +39376,22 @@
     </row>
     <row r="3056">
       <c r="AU3056" t="s" s="0">
-        <v>795</v>
+        <v>3924</v>
       </c>
     </row>
     <row r="3057">
       <c r="AU3057" t="s" s="0">
-        <v>3924</v>
+        <v>3925</v>
       </c>
     </row>
     <row r="3058">
       <c r="AU3058" t="s" s="0">
-        <v>3925</v>
+        <v>3926</v>
       </c>
     </row>
     <row r="3059">
       <c r="AU3059" t="s" s="0">
-        <v>3926</v>
+        <v>795</v>
       </c>
     </row>
     <row r="3060">
@@ -43885,7 +43909,47 @@
         <v>4829</v>
       </c>
     </row>
-    <row r="3963"/>
+    <row r="3963">
+      <c r="AU3963" t="s" s="0">
+        <v>4830</v>
+      </c>
+    </row>
+    <row r="3964">
+      <c r="AU3964" t="s" s="0">
+        <v>4831</v>
+      </c>
+    </row>
+    <row r="3965">
+      <c r="AU3965" t="s" s="0">
+        <v>4832</v>
+      </c>
+    </row>
+    <row r="3966">
+      <c r="AU3966" t="s" s="0">
+        <v>4833</v>
+      </c>
+    </row>
+    <row r="3967">
+      <c r="AU3967" t="s" s="0">
+        <v>4834</v>
+      </c>
+    </row>
+    <row r="3968">
+      <c r="AU3968" t="s" s="0">
+        <v>4835</v>
+      </c>
+    </row>
+    <row r="3969">
+      <c r="AU3969" t="s" s="0">
+        <v>4836</v>
+      </c>
+    </row>
+    <row r="3970">
+      <c r="AU3970" t="s" s="0">
+        <v>4837</v>
+      </c>
+    </row>
+    <row r="3971"/>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -43952,13 +44016,13 @@
   <sheetData>
     <row r="1" ht="50.0" customHeight="true">
       <c r="A1" t="s" s="42">
-        <v>4830</v>
+        <v>4838</v>
       </c>
       <c r="B1" s="42"/>
       <c r="C1" s="42"/>
       <c r="D1" s="42"/>
       <c r="E1" t="s" s="42">
-        <v>4830</v>
+        <v>4838</v>
       </c>
       <c r="F1" s="42"/>
       <c r="G1" s="42"/>
@@ -44010,323 +44074,323 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="42">
-        <v>4831</v>
+        <v>4839</v>
       </c>
       <c r="B2" t="s" s="48">
-        <v>4832</v>
+        <v>4840</v>
       </c>
       <c r="C2" t="s" s="48">
-        <v>4832</v>
+        <v>4840</v>
       </c>
       <c r="D2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="E2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="F2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="G2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="H2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="I2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="J2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="K2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="L2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="M2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="N2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="O2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="P2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="Q2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="R2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="S2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="T2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="U2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="V2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="W2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="X2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="Y2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="Z2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AA2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AB2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AC2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AD2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AE2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AF2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AG2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AH2" t="s" s="43">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AI2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AJ2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AK2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AL2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AM2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AN2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AO2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AP2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AQ2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AR2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AS2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AT2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AU2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AV2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AW2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AX2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AY2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AZ2" t="s" s="44">
-        <v>4834</v>
+        <v>4842</v>
       </c>
     </row>
     <row r="3" ht="210.0" customHeight="true">
       <c r="A3" t="s" s="42">
-        <v>4835</v>
+        <v>4843</v>
       </c>
       <c r="B3" t="s" s="46">
-        <v>4837</v>
+        <v>4845</v>
       </c>
       <c r="C3" t="s" s="46">
-        <v>4838</v>
+        <v>4846</v>
       </c>
       <c r="D3" t="s" s="46">
-        <v>4839</v>
+        <v>4847</v>
       </c>
       <c r="E3" t="s" s="46">
-        <v>4840</v>
+        <v>4848</v>
       </c>
       <c r="F3" t="s" s="46">
-        <v>4841</v>
+        <v>4849</v>
       </c>
       <c r="G3" t="s" s="46">
-        <v>4842</v>
+        <v>4850</v>
       </c>
       <c r="H3" t="s" s="46">
-        <v>4844</v>
+        <v>4852</v>
       </c>
       <c r="I3" t="s" s="46">
-        <v>4845</v>
+        <v>4853</v>
       </c>
       <c r="J3" t="s" s="46">
-        <v>4846</v>
+        <v>4854</v>
       </c>
       <c r="K3" t="s" s="46">
-        <v>4847</v>
+        <v>4855</v>
       </c>
       <c r="L3" t="s" s="46">
-        <v>4848</v>
+        <v>4856</v>
       </c>
       <c r="M3" t="s" s="46">
-        <v>4849</v>
+        <v>4857</v>
       </c>
       <c r="N3" t="s" s="46">
-        <v>4850</v>
+        <v>4858</v>
       </c>
       <c r="O3" t="s" s="46">
-        <v>4851</v>
+        <v>4859</v>
       </c>
       <c r="P3" t="s" s="46">
-        <v>4852</v>
+        <v>4860</v>
       </c>
       <c r="Q3" t="s" s="46">
-        <v>4853</v>
+        <v>4861</v>
       </c>
       <c r="R3" t="s" s="46">
-        <v>4854</v>
+        <v>4862</v>
       </c>
       <c r="S3" t="s" s="46">
-        <v>4855</v>
+        <v>4863</v>
       </c>
       <c r="T3" t="s" s="46">
-        <v>4856</v>
+        <v>4864</v>
       </c>
       <c r="U3" t="s" s="46">
-        <v>4857</v>
+        <v>4865</v>
       </c>
       <c r="V3" t="s" s="46">
-        <v>4858</v>
+        <v>4866</v>
       </c>
       <c r="W3" t="s" s="46">
-        <v>4859</v>
+        <v>4867</v>
       </c>
       <c r="X3" t="s" s="46">
-        <v>4860</v>
+        <v>4868</v>
       </c>
       <c r="Y3" t="s" s="46">
-        <v>4861</v>
+        <v>4869</v>
       </c>
       <c r="Z3" t="s" s="46">
-        <v>4862</v>
+        <v>4870</v>
       </c>
       <c r="AA3" t="s" s="46">
-        <v>4863</v>
+        <v>4871</v>
       </c>
       <c r="AB3" t="s" s="46">
-        <v>4864</v>
+        <v>4872</v>
       </c>
       <c r="AC3" t="s" s="46">
-        <v>4865</v>
+        <v>4873</v>
       </c>
       <c r="AD3" t="s" s="46">
-        <v>4866</v>
+        <v>4874</v>
       </c>
       <c r="AE3" t="s" s="46">
-        <v>4867</v>
+        <v>4875</v>
       </c>
       <c r="AF3" t="s" s="46">
-        <v>4868</v>
+        <v>4876</v>
       </c>
       <c r="AG3" t="s" s="46">
-        <v>4869</v>
+        <v>4877</v>
       </c>
       <c r="AH3" t="s" s="46">
-        <v>4870</v>
+        <v>4878</v>
       </c>
       <c r="AI3" t="s" s="46">
-        <v>4871</v>
+        <v>4879</v>
       </c>
       <c r="AJ3" t="s" s="46">
-        <v>4872</v>
+        <v>4880</v>
       </c>
       <c r="AK3" t="s" s="46">
-        <v>4873</v>
+        <v>4881</v>
       </c>
       <c r="AL3" t="s" s="46">
-        <v>4874</v>
+        <v>4882</v>
       </c>
       <c r="AM3" t="s" s="46">
-        <v>4875</v>
+        <v>4883</v>
       </c>
       <c r="AN3" t="s" s="46">
-        <v>4876</v>
+        <v>4884</v>
       </c>
       <c r="AO3" t="s" s="46">
-        <v>4877</v>
+        <v>4885</v>
       </c>
       <c r="AP3" t="s" s="46">
-        <v>4878</v>
+        <v>4886</v>
       </c>
       <c r="AQ3" t="s" s="46">
-        <v>4879</v>
+        <v>4887</v>
       </c>
       <c r="AR3" t="s" s="46">
-        <v>4880</v>
+        <v>4888</v>
       </c>
       <c r="AS3" t="s" s="46">
-        <v>4881</v>
+        <v>4889</v>
       </c>
       <c r="AT3" t="s" s="46">
-        <v>4882</v>
+        <v>4890</v>
       </c>
       <c r="AU3" t="s" s="46">
-        <v>4883</v>
+        <v>4891</v>
       </c>
       <c r="AV3" t="s" s="46">
-        <v>4884</v>
+        <v>4892</v>
       </c>
       <c r="AW3" t="s" s="46">
-        <v>4885</v>
+        <v>4893</v>
       </c>
       <c r="AX3" t="s" s="46">
-        <v>4886</v>
+        <v>4894</v>
       </c>
       <c r="AY3" t="s" s="46">
-        <v>4887</v>
+        <v>4895</v>
       </c>
       <c r="AZ3" t="s" s="46">
-        <v>4888</v>
+        <v>4896</v>
       </c>
     </row>
     <row r="4" ht="40.0" customHeight="true">
       <c r="A4" t="s" s="42">
-        <v>4836</v>
+        <v>4844</v>
       </c>
       <c r="B4" s="42"/>
       <c r="C4" s="42"/>
@@ -44334,7 +44398,7 @@
       <c r="E4" s="45"/>
       <c r="F4" s="42"/>
       <c r="G4" s="45" t="s">
-        <v>4843</v>
+        <v>4851</v>
       </c>
       <c r="H4" s="42"/>
       <c r="I4" s="45"/>
@@ -44363,14 +44427,14 @@
       <c r="AF4" s="45"/>
       <c r="AG4" s="45"/>
       <c r="AH4" s="45" t="s">
-        <v>4843</v>
+        <v>4851</v>
       </c>
       <c r="AI4" s="42"/>
       <c r="AJ4" s="42"/>
       <c r="AK4" s="42"/>
       <c r="AL4" s="42"/>
       <c r="AM4" s="45" t="s">
-        <v>4843</v>
+        <v>4851</v>
       </c>
       <c r="AN4" s="42"/>
       <c r="AO4" s="45"/>
@@ -44388,7 +44452,7 @@
     </row>
     <row r="5">
       <c r="D5" t="s" s="51">
-        <v>4889</v>
+        <v>4897</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>157</v>
@@ -44430,13 +44494,13 @@
         <v>263</v>
       </c>
       <c r="AH5" t="s">
-        <v>4891</v>
+        <v>4899</v>
       </c>
       <c r="AL5" t="s">
-        <v>4890</v>
+        <v>4898</v>
       </c>
       <c r="AM5" t="s">
-        <v>4890</v>
+        <v>4898</v>
       </c>
       <c r="AQ5" t="s">
         <v>306</v>
@@ -44453,7 +44517,7 @@
     </row>
     <row r="6">
       <c r="D6" t="s" s="51">
-        <v>4889</v>
+        <v>4897</v>
       </c>
       <c r="E6" t="s" s="0">
         <v>157</v>
@@ -44495,13 +44559,13 @@
         <v>263</v>
       </c>
       <c r="AH6" t="s">
-        <v>4893</v>
+        <v>4901</v>
       </c>
       <c r="AL6" t="s">
-        <v>4892</v>
+        <v>4900</v>
       </c>
       <c r="AM6" t="s">
-        <v>4892</v>
+        <v>4900</v>
       </c>
       <c r="AQ6" t="s">
         <v>227</v>
@@ -44518,7 +44582,7 @@
     </row>
     <row r="7">
       <c r="D7" t="s" s="51">
-        <v>4889</v>
+        <v>4897</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>157</v>
@@ -44560,13 +44624,13 @@
         <v>263</v>
       </c>
       <c r="AH7" t="s">
-        <v>4895</v>
+        <v>4903</v>
       </c>
       <c r="AL7" t="s">
-        <v>4894</v>
+        <v>4902</v>
       </c>
       <c r="AM7" t="s">
-        <v>4894</v>
+        <v>4902</v>
       </c>
       <c r="AQ7" t="s">
         <v>367</v>
@@ -50930,7 +50994,7 @@
       <formula1>'Validation Sheet'!$AT$3:$AT$6</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AU5:AU305" allowBlank="true" errorStyle="stop" showErrorMessage="true" errorTitle="Invalid value" error="Please select a value from the dropdown only" promptTitle="Hint key" prompt="Please select a value from the dropdown only" showInputMessage="true">
-      <formula1>'Validation Sheet'!$AU$3:$AU$3962</formula1>
+      <formula1>'Validation Sheet'!$AU$3:$AU$3970</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AV5:AV305" allowBlank="true" errorStyle="stop" showErrorMessage="true" errorTitle="Invalid value" error="Please select a value from the dropdown only" promptTitle="Hint key" prompt="Please select a value from the dropdown only" showInputMessage="true">
       <formula1>'Validation Sheet'!$AV$3:$AV$4</formula1>
@@ -51044,13 +51108,13 @@
   <sheetData>
     <row r="1" ht="50.0" customHeight="true">
       <c r="A1" t="s" s="70">
-        <v>4830</v>
+        <v>4838</v>
       </c>
       <c r="B1" s="70"/>
       <c r="C1" s="70"/>
       <c r="D1" s="70"/>
       <c r="E1" t="s" s="70">
-        <v>4830</v>
+        <v>4838</v>
       </c>
       <c r="F1" s="70"/>
       <c r="G1" s="70"/>
@@ -51102,323 +51166,323 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="70">
-        <v>4831</v>
+        <v>4839</v>
       </c>
       <c r="B2" t="s" s="76">
-        <v>4832</v>
+        <v>4840</v>
       </c>
       <c r="C2" t="s" s="76">
-        <v>4832</v>
+        <v>4840</v>
       </c>
       <c r="D2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="E2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="F2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="G2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="H2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="I2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="J2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="K2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="L2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="M2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="N2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="O2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="P2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="Q2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="R2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="S2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="T2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="U2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="V2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="W2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="X2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="Y2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="Z2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AA2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AB2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AC2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AD2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AE2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AF2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AG2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AH2" t="s" s="71">
-        <v>4833</v>
+        <v>4841</v>
       </c>
       <c r="AI2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AJ2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AK2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AL2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AM2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AN2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AO2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AP2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AQ2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AR2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AS2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AT2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AU2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AV2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AW2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AX2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AY2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
       <c r="AZ2" t="s" s="72">
-        <v>4834</v>
+        <v>4842</v>
       </c>
     </row>
     <row r="3" ht="210.0" customHeight="true">
       <c r="A3" t="s" s="70">
-        <v>4835</v>
+        <v>4843</v>
       </c>
       <c r="B3" t="s" s="74">
-        <v>4837</v>
+        <v>4845</v>
       </c>
       <c r="C3" t="s" s="74">
-        <v>4838</v>
+        <v>4846</v>
       </c>
       <c r="D3" t="s" s="74">
-        <v>4839</v>
+        <v>4847</v>
       </c>
       <c r="E3" t="s" s="74">
-        <v>4840</v>
+        <v>4848</v>
       </c>
       <c r="F3" t="s" s="74">
-        <v>4841</v>
+        <v>4849</v>
       </c>
       <c r="G3" t="s" s="74">
-        <v>4842</v>
+        <v>4850</v>
       </c>
       <c r="H3" t="s" s="74">
-        <v>4844</v>
+        <v>4852</v>
       </c>
       <c r="I3" t="s" s="74">
-        <v>4845</v>
+        <v>4853</v>
       </c>
       <c r="J3" t="s" s="74">
-        <v>4846</v>
+        <v>4854</v>
       </c>
       <c r="K3" t="s" s="74">
-        <v>4847</v>
+        <v>4855</v>
       </c>
       <c r="L3" t="s" s="74">
-        <v>4848</v>
+        <v>4856</v>
       </c>
       <c r="M3" t="s" s="74">
-        <v>4849</v>
+        <v>4857</v>
       </c>
       <c r="N3" t="s" s="74">
-        <v>4850</v>
+        <v>4858</v>
       </c>
       <c r="O3" t="s" s="74">
-        <v>4851</v>
+        <v>4859</v>
       </c>
       <c r="P3" t="s" s="74">
-        <v>4852</v>
+        <v>4860</v>
       </c>
       <c r="Q3" t="s" s="74">
-        <v>4853</v>
+        <v>4861</v>
       </c>
       <c r="R3" t="s" s="74">
-        <v>4854</v>
+        <v>4862</v>
       </c>
       <c r="S3" t="s" s="74">
-        <v>4855</v>
+        <v>4863</v>
       </c>
       <c r="T3" t="s" s="74">
-        <v>4856</v>
+        <v>4864</v>
       </c>
       <c r="U3" t="s" s="74">
-        <v>4857</v>
+        <v>4865</v>
       </c>
       <c r="V3" t="s" s="74">
-        <v>4858</v>
+        <v>4866</v>
       </c>
       <c r="W3" t="s" s="74">
-        <v>4859</v>
+        <v>4867</v>
       </c>
       <c r="X3" t="s" s="74">
-        <v>4860</v>
+        <v>4868</v>
       </c>
       <c r="Y3" t="s" s="74">
-        <v>4861</v>
+        <v>4869</v>
       </c>
       <c r="Z3" t="s" s="74">
-        <v>4862</v>
+        <v>4870</v>
       </c>
       <c r="AA3" t="s" s="74">
-        <v>4863</v>
+        <v>4871</v>
       </c>
       <c r="AB3" t="s" s="74">
-        <v>4864</v>
+        <v>4872</v>
       </c>
       <c r="AC3" t="s" s="74">
-        <v>4865</v>
+        <v>4873</v>
       </c>
       <c r="AD3" t="s" s="74">
-        <v>4866</v>
+        <v>4874</v>
       </c>
       <c r="AE3" t="s" s="74">
-        <v>4867</v>
+        <v>4875</v>
       </c>
       <c r="AF3" t="s" s="74">
-        <v>4868</v>
+        <v>4876</v>
       </c>
       <c r="AG3" t="s" s="74">
-        <v>4869</v>
+        <v>4877</v>
       </c>
       <c r="AH3" t="s" s="74">
-        <v>4870</v>
+        <v>4878</v>
       </c>
       <c r="AI3" t="s" s="74">
-        <v>4871</v>
+        <v>4879</v>
       </c>
       <c r="AJ3" t="s" s="74">
-        <v>4872</v>
+        <v>4880</v>
       </c>
       <c r="AK3" t="s" s="74">
-        <v>4873</v>
+        <v>4881</v>
       </c>
       <c r="AL3" t="s" s="74">
-        <v>4874</v>
+        <v>4882</v>
       </c>
       <c r="AM3" t="s" s="74">
-        <v>4875</v>
+        <v>4883</v>
       </c>
       <c r="AN3" t="s" s="74">
-        <v>4876</v>
+        <v>4884</v>
       </c>
       <c r="AO3" t="s" s="74">
-        <v>4877</v>
+        <v>4885</v>
       </c>
       <c r="AP3" t="s" s="74">
-        <v>4878</v>
+        <v>4886</v>
       </c>
       <c r="AQ3" t="s" s="74">
-        <v>4879</v>
+        <v>4887</v>
       </c>
       <c r="AR3" t="s" s="74">
-        <v>4880</v>
+        <v>4888</v>
       </c>
       <c r="AS3" t="s" s="74">
-        <v>4881</v>
+        <v>4889</v>
       </c>
       <c r="AT3" t="s" s="74">
-        <v>4882</v>
+        <v>4890</v>
       </c>
       <c r="AU3" t="s" s="74">
-        <v>4883</v>
+        <v>4891</v>
       </c>
       <c r="AV3" t="s" s="74">
-        <v>4884</v>
+        <v>4892</v>
       </c>
       <c r="AW3" t="s" s="74">
-        <v>4885</v>
+        <v>4893</v>
       </c>
       <c r="AX3" t="s" s="74">
-        <v>4886</v>
+        <v>4894</v>
       </c>
       <c r="AY3" t="s" s="74">
-        <v>4887</v>
+        <v>4895</v>
       </c>
       <c r="AZ3" t="s" s="74">
-        <v>4888</v>
+        <v>4896</v>
       </c>
     </row>
     <row r="4" ht="40.0" customHeight="true">
       <c r="A4" t="s" s="70">
-        <v>4836</v>
+        <v>4844</v>
       </c>
       <c r="B4" s="70"/>
       <c r="C4" s="70"/>
@@ -51426,7 +51490,7 @@
       <c r="E4" s="73"/>
       <c r="F4" s="70"/>
       <c r="G4" s="73" t="s">
-        <v>4843</v>
+        <v>4851</v>
       </c>
       <c r="H4" s="70"/>
       <c r="I4" s="73"/>
@@ -51455,14 +51519,14 @@
       <c r="AF4" s="73"/>
       <c r="AG4" s="73"/>
       <c r="AH4" s="73" t="s">
-        <v>4843</v>
+        <v>4851</v>
       </c>
       <c r="AI4" s="70"/>
       <c r="AJ4" s="70"/>
       <c r="AK4" s="70"/>
       <c r="AL4" s="70"/>
       <c r="AM4" s="73" t="s">
-        <v>4843</v>
+        <v>4851</v>
       </c>
       <c r="AN4" s="70"/>
       <c r="AO4" s="73"/>
@@ -57869,7 +57933,7 @@
       <formula1>'Validation Sheet'!$AT$3:$AT$6</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AU5:AU305" allowBlank="true" errorStyle="stop" showErrorMessage="true" errorTitle="Invalid value" error="Please select a value from the dropdown only" promptTitle="Hint key" prompt="Please select a value from the dropdown only" showInputMessage="true">
-      <formula1>'Validation Sheet'!$AU$3:$AU$3962</formula1>
+      <formula1>'Validation Sheet'!$AU$3:$AU$3970</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="AV5:AV305" allowBlank="true" errorStyle="stop" showErrorMessage="true" errorTitle="Invalid value" error="Please select a value from the dropdown only" promptTitle="Hint key" prompt="Please select a value from the dropdown only" showInputMessage="true">
       <formula1>'Validation Sheet'!$AV$3:$AV$4</formula1>

</xml_diff>